<commit_message>
salvando de qualquer jeito so por conta da queda de luz
</commit_message>
<xml_diff>
--- a/resumos.xlsx
+++ b/resumos.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -459,10 +459,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>https://grownt.tech/recursos-publicos-para-inovacao-quais-empresas-podem-acessar-entenda-criterios-porte-e-setores-prioritarios/</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Recursos públicos para inovação são instrumentos de fomento oferecidos por órgãos como Finep, BNDES, Embrapii, Sebrae, agências estaduais e fundos setoriais, para apoiar projetos de pesquisa, desenvolvimento e inovação (PD&amp;I) em empresas. Esses recursos podem aparecer como:  Na prática, esses mecanismos servem para dividir risco e investimento entre empresa e governo em projetos com potencial de impacto tecnológico e econômico. De forma geral, podem acessar esses instrumentos:  Além disso, muitos programas exigem que a empresa:  Existe um conjunto relevante de programas desenhados para MEI, micro e pequenas empresas, frequentemente com:  Exemplo: a parceria Embrapii–Sebrae oferece até 90% de apoio técnico e financeiro para projetos de inovação de micro e pequenas empresas com faturamento até R$ 4,8 milhões ao ano. Em chamadas específicas, MEI, microempresas e empresas de pequeno porte podem se inscrever diretamente em projetos de inovação apoiados por Embrapii e Sebrae. Médias empresas são bastante relevantes no mapa de fomento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>https://www.financiamentodainovacao.com.br/editais-em-aberto/</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Confira abaixo os editais que estão abertos no momento. Descritivo: Incentivo em Pesquisa Inovativa em Pequenas Empresas com potencial mercadológico. Fase 1: Estudo/Análise de Viabilidade Técnico-científica da pesquisa; Fase 2:Desenvolvimento da pesquisa técnico-cientifica; Fase 3: Desenvolvimento comercial e industrial do produto/serviço. Valor do Edital:
 Fase 1 – R$ 300 mil
@@ -471,27 +483,28 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>https://www.conjur.com.br/2025-ago-26/politicas-publicas-e-instrumentos-de-fomento-a-inovacao-portuaria/</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>,  26 de agosto de 2025, 9h24 Na coluna anterior, analisamos a evolução regulatória do setor portuário, da gestão estatal centralizada a um modelo mais competitivo e aberto à inovação. A legislação das décadas de 1990 e 2010, ao ampliar a participação privada e redefinir o papel das autoridades portuárias, criou condições favoráveis ao surgimento de ecossistemas inovadores. Claudio Neves/Portos do Paraná Agora, o foco recai sobre os instrumentos de fomento disponíveis para impulsionar a inovação portuária. O objetivo é mostrar como incentivos tributários, crédito público, mecanismos regulatórios e cláusulas contratuais podem ser articulados em uma estratégia integrada que fortaleça a autonomia tecnológica, reduza a dependência externa e amplie a competitividade. Ao deslocar o foco do panorama histórico-regulatório para os instrumentos jurídicos e econômicos específicos, pretende-se avaliar em que medida o Brasil dispõe de um arcabouço normativo e institucional sólido para sustentar uma política consistente de modernização portuária, alinhada às exigências globais de eficiência, sustentabilidade e segurança.</t>
-        </is>
-      </c>
-    </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://ddtax.com.br/2025/08/29/politicas-publicas-e-instrumentos-de-fomento-a-inovacao-portuaria/</t>
+          <t>https://apet.org.br/artigos/politicas-publicas-e-instrumentos-de-fomento-a-inovacao-portuaria/</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Na coluna anterior, analisamos a evolução regulatória do setor portuário, da gestão estatal centralizada a um modelo mais competitivo e aberto à inovação. A legislação das décadas de 1990 e 2010, ao ampliar a participação privada e redefinir o papel das autoridades portuárias, criou condições favoráveis ao surgimento de ecossistemas inovadores. Agora, o foco recai sobre os instrumentos de fomento disponíveis para impulsionar a inovação portuária. O objetivo é mostrar como incentivos tributários, crédito público, mecanismos regulatórios e cláusulas contratuais podem ser articulados em uma estratégia integrada que fortaleça a autonomia tecnológica, reduza a dependência externa e amplie a competitividade. Ao deslocar o foco do panorama histórico-regulatório para os instrumentos jurídicos e econômicos específicos, pretende-se avaliar em que medida o Brasil dispõe de um arcabouço normativo e institucional sólido para sustentar uma política consistente de modernização portuária, alinhada às exigências globais de eficiência, sustentabilidade e segurança.</t>
+          <t>26/08/2025 12:00 am Na coluna anterior, analisamos a evolução regulatória do setor portuário, da gestão estatal centralizada a um modelo mais competitivo e aberto à inovação. A legislação das décadas de 1990 e 2010, ao ampliar a participação privada e redefinir o papel das autoridades portuárias, criou condições favoráveis ao surgimento de ecossistemas inovadores. Claudio Neves/Portos do Paranáporto portuários trabalhadores
+Agora, o foco recai sobre os instrumentos de fomento disponíveis para impulsionar a inovação portuária. O objetivo é mostrar como incentivos tributários, crédito público, mecanismos regulatórios e cláusulas contratuais podem ser articulados em uma estratégia integrada que fortaleça a autonomia tecnológica, reduza a dependência externa e amplie a competitividade. Ao deslocar o foco do panorama histórico-regulatório para os instrumentos jurídicos e econômicos específicos, pretende-se avaliar em que medida o Brasil dispõe de um arcabouço normativo e institucional sólido para sustentar uma política consistente de modernização portuária, alinhada às exigências globais de eficiência, sustentabilidade e segurança.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>https://www.conjur.com.br/2025-ago-26/politicas-publicas-e-instrumentos-de-fomento-a-inovacao-portuaria/</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>,  26 de agosto de 2025, 9h24 Na coluna anterior, analisamos a evolução regulatória do setor portuário, da gestão estatal centralizada a um modelo mais competitivo e aberto à inovação. A legislação das décadas de 1990 e 2010, ao ampliar a participação privada e redefinir o papel das autoridades portuárias, criou condições favoráveis ao surgimento de ecossistemas inovadores. Claudio Neves/Portos do Paraná Agora, o foco recai sobre os instrumentos de fomento disponíveis para impulsionar a inovação portuária. O objetivo é mostrar como incentivos tributários, crédito público, mecanismos regulatórios e cláusulas contratuais podem ser articulados em uma estratégia integrada que fortaleça a autonomia tecnológica, reduza a dependência externa e amplie a competitividade. Ao deslocar o foco do panorama histórico-regulatório para os instrumentos jurídicos e econômicos específicos, pretende-se avaliar em que medida o Brasil dispõe de um arcabouço normativo e institucional sólido para sustentar uma política consistente de modernização portuária, alinhada às exigências globais de eficiência, sustentabilidade e segurança.</t>
         </is>
       </c>
     </row>

</xml_diff>